<commit_message>
Sync football model artifacts 2026-05-23
</commit_message>
<xml_diff>
--- a/data/exports/football-recap-master.xlsx
+++ b/data/exports/football-recap-master.xlsx
@@ -8083,44 +8083,44 @@
         </is>
       </c>
       <c r="K79">
-        <v>0.4032</v>
+        <v>0.3836</v>
       </c>
       <c r="L79">
-        <v>0.3008</v>
+        <v>0.3107</v>
       </c>
       <c r="M79">
-        <v>0.2961</v>
+        <v>0.3057</v>
       </c>
       <c r="N79">
-        <v>0.4032</v>
+        <v>0.3836</v>
       </c>
       <c r="O79">
-        <v>0.3008</v>
+        <v>0.3107</v>
       </c>
       <c r="P79">
-        <v>0.2961</v>
+        <v>0.3057</v>
       </c>
       <c r="Q79">
-        <v>0.4666</v>
+        <v>0.4418</v>
       </c>
       <c r="R79">
-        <v>0.2588</v>
+        <v>0.2611</v>
       </c>
       <c r="S79">
-        <v>0.2747</v>
+        <v>0.2972</v>
       </c>
       <c r="T79" t="inlineStr">
         <is>
-          <t>1-1:12.3% / 1-0:10.6% / 2-1:9.2%</t>
+          <t>1-1:12.5% / 1-0:10.7% / 2-1:9%</t>
         </is>
       </c>
       <c r="U79" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>高</t>
         </is>
       </c>
       <c r="V79">
-        <v>31.25</v>
+        <v>25.43</v>
       </c>
       <c r="W79" t="inlineStr">
         <is>
@@ -8135,7 +8135,7 @@
       </c>
       <c r="Z79" t="inlineStr">
         <is>
-          <t>经模型综合分析：澳超，主胜概率领先平局；风险中；已接入本次实时赔率快照，并完成隐含概率换算与高级数据修正</t>
+          <t>经模型综合分析：澳超，主胜概率领先平局；风险高；已接入本次实时赔率快照，并完成隐含概率换算与高级数据修正</t>
         </is>
       </c>
       <c r="AA79" t="inlineStr">
@@ -11744,42 +11744,42 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>客胜</t>
+          <t>主胜</t>
         </is>
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>主胜</t>
+          <t>平局</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>2-0</t>
         </is>
       </c>
       <c r="H109" t="inlineStr">
         <is>
-          <t>2-1</t>
+          <t>2-2</t>
         </is>
       </c>
       <c r="I109" t="inlineStr">
         <is>
-          <t>平局-客胜</t>
+          <t>主胜-主胜</t>
         </is>
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>客胜-主胜</t>
+          <t>主胜-平局</t>
         </is>
       </c>
       <c r="K109">
-        <v>0.2543</v>
+        <v>0.7045</v>
       </c>
       <c r="L109">
-        <v>0.2447</v>
+        <v>0.1655</v>
       </c>
       <c r="M109">
-        <v>0.501</v>
+        <v>0.13</v>
       </c>
       <c r="N109">
         <v>0.2543</v>
@@ -11810,7 +11810,7 @@
         </is>
       </c>
       <c r="V109">
-        <v>48.48</v>
+        <v>92.23</v>
       </c>
       <c r="W109" t="inlineStr">
         <is>
@@ -11825,7 +11825,7 @@
       </c>
       <c r="Z109" t="inlineStr">
         <is>
-          <t>经模型综合分析：德国杯，客胜概率领先主胜；风险中；已接入本次实时赔率快照，并完成隐含概率换算与高级数据修正</t>
+          <t>经模型综合分析：德国杯，客胜概率领先主胜；风险中；已接入本次实时赔率快照，并完成隐含概率换算与高级数据修正；同场次已与竞彩足球 周六014 胜平负方向强制一致</t>
         </is>
       </c>
       <c r="AA109" t="inlineStr">
@@ -11867,42 +11867,42 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
+          <t>客胜</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
           <t>主胜</t>
         </is>
       </c>
-      <c r="F110" t="inlineStr">
-        <is>
-          <t>平局</t>
-        </is>
-      </c>
       <c r="G110" t="inlineStr">
         <is>
-          <t>2-0</t>
+          <t>1-2</t>
         </is>
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>1-1</t>
+          <t>2-1</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>主胜-主胜</t>
+          <t>主胜-客胜</t>
         </is>
       </c>
       <c r="J110" t="inlineStr">
         <is>
-          <t>平局-平局</t>
+          <t>客胜-主胜</t>
         </is>
       </c>
       <c r="K110">
-        <v>0.627</v>
+        <v>0.2785</v>
       </c>
       <c r="L110">
-        <v>0.2197</v>
+        <v>0.253</v>
       </c>
       <c r="M110">
-        <v>0.1532</v>
+        <v>0.4685</v>
       </c>
       <c r="N110">
         <v>0.627</v>
@@ -11933,7 +11933,7 @@
         </is>
       </c>
       <c r="V110">
-        <v>72</v>
+        <v>42.08</v>
       </c>
       <c r="W110" t="inlineStr">
         <is>
@@ -11948,7 +11948,7 @@
       </c>
       <c r="Z110" t="inlineStr">
         <is>
-          <t>经模型综合分析：意甲，主胜概率领先平局；风险中；已接入本次实时赔率快照，并完成隐含概率换算与高级数据修正</t>
+          <t>经模型综合分析：意甲，主胜概率领先平局；风险中；已接入本次实时赔率快照，并完成隐含概率换算与高级数据修正；同场次已与竞彩足球 周六013 胜平负方向强制一致</t>
         </is>
       </c>
       <c r="AA110" t="inlineStr">
@@ -12000,7 +12000,7 @@
       </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>2-1</t>
+          <t>3-1</t>
         </is>
       </c>
       <c r="H111" t="inlineStr">
@@ -12019,13 +12019,13 @@
         </is>
       </c>
       <c r="K111">
-        <v>0.4947</v>
+        <v>0.6014</v>
       </c>
       <c r="L111">
-        <v>0.2664</v>
+        <v>0.2297</v>
       </c>
       <c r="M111">
-        <v>0.239</v>
+        <v>0.1689</v>
       </c>
       <c r="N111">
         <v>0.4947</v>
@@ -12056,7 +12056,7 @@
         </is>
       </c>
       <c r="V111">
-        <v>46.37</v>
+        <v>69.75</v>
       </c>
       <c r="W111" t="inlineStr">
         <is>
@@ -12071,7 +12071,7 @@
       </c>
       <c r="Z111" t="inlineStr">
         <is>
-          <t>经模型综合分析：意甲，主胜概率领先平局；风险中；已接入本次实时赔率快照，并完成隐含概率换算与高级数据修正</t>
+          <t>经模型综合分析：意甲，主胜概率领先平局；风险中；已接入本次实时赔率快照，并完成隐含概率换算与高级数据修正；同场次已与竞彩足球 周六016 胜平负方向强制一致</t>
         </is>
       </c>
       <c r="AA111" t="inlineStr">
@@ -12128,7 +12128,7 @@
       </c>
       <c r="H112" t="inlineStr">
         <is>
-          <t>1-1</t>
+          <t>2-2</t>
         </is>
       </c>
       <c r="I112" t="inlineStr">
@@ -12142,13 +12142,13 @@
         </is>
       </c>
       <c r="K112">
-        <v>0.3949</v>
+        <v>0.5438</v>
       </c>
       <c r="L112">
-        <v>0.3331</v>
+        <v>0.2578</v>
       </c>
       <c r="M112">
-        <v>0.272</v>
+        <v>0.1984</v>
       </c>
       <c r="N112">
         <v>0.3949</v>
@@ -12175,11 +12175,11 @@
       </c>
       <c r="U112" t="inlineStr">
         <is>
-          <t>高</t>
+          <t>中</t>
         </is>
       </c>
       <c r="V112">
-        <v>22.44</v>
+        <v>57.89</v>
       </c>
       <c r="W112" t="inlineStr">
         <is>
@@ -12194,7 +12194,7 @@
       </c>
       <c r="Z112" t="inlineStr">
         <is>
-          <t>经模型综合分析：西甲，主胜概率领先平局；风险高；已接入本次实时赔率快照，并完成隐含概率换算与高级数据修正</t>
+          <t>经模型综合分析：西甲，主胜概率领先平局；风险高；已接入本次实时赔率快照，并完成隐含概率换算与高级数据修正；同场次已与竞彩足球 周六022 胜平负方向强制一致</t>
         </is>
       </c>
       <c r="AA112" t="inlineStr">
@@ -12251,7 +12251,7 @@
       </c>
       <c r="H113" t="inlineStr">
         <is>
-          <t>1-1</t>
+          <t>0-0</t>
         </is>
       </c>
       <c r="I113" t="inlineStr">
@@ -12265,13 +12265,13 @@
         </is>
       </c>
       <c r="K113">
-        <v>0.5101</v>
+        <v>0.3719</v>
       </c>
       <c r="L113">
-        <v>0.2496</v>
+        <v>0.3471</v>
       </c>
       <c r="M113">
-        <v>0.2402</v>
+        <v>0.281</v>
       </c>
       <c r="N113">
         <v>0.5101</v>
@@ -12298,11 +12298,11 @@
       </c>
       <c r="U113" t="inlineStr">
         <is>
-          <t>中</t>
+          <t>高</t>
         </is>
       </c>
       <c r="V113">
-        <v>50.37</v>
+        <v>18.51</v>
       </c>
       <c r="W113" t="inlineStr">
         <is>
@@ -12317,7 +12317,7 @@
       </c>
       <c r="Z113" t="inlineStr">
         <is>
-          <t>经模型综合分析：西甲，主胜概率领先平局；风险中；已接入本次实时赔率快照，并完成隐含概率换算与高级数据修正</t>
+          <t>经模型综合分析：西甲，主胜概率领先平局；风险中；已接入本次实时赔率快照，并完成隐含概率换算与高级数据修正；同场次已与竞彩足球 周六021 胜平负方向强制一致</t>
         </is>
       </c>
       <c r="AA113" t="inlineStr">
@@ -12364,7 +12364,7 @@
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>客胜</t>
+          <t>平局</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
@@ -12374,7 +12374,7 @@
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>1-1</t>
         </is>
       </c>
       <c r="I114" t="inlineStr">
@@ -12384,17 +12384,17 @@
       </c>
       <c r="J114" t="inlineStr">
         <is>
-          <t>平局-客胜</t>
+          <t>平局-平局</t>
         </is>
       </c>
       <c r="K114">
-        <v>0.4605</v>
+        <v>0.5348</v>
       </c>
       <c r="L114">
-        <v>0.2536</v>
+        <v>0.2446</v>
       </c>
       <c r="M114">
-        <v>0.2859</v>
+        <v>0.2206</v>
       </c>
       <c r="N114">
         <v>0.4605</v>
@@ -12425,7 +12425,7 @@
         </is>
       </c>
       <c r="V114">
-        <v>39.07</v>
+        <v>57.62</v>
       </c>
       <c r="W114" t="inlineStr">
         <is>
@@ -12440,7 +12440,7 @@
       </c>
       <c r="Z114" t="inlineStr">
         <is>
-          <t>经模型综合分析：西甲，主胜概率领先客胜；风险中；已接入本次实时赔率快照，并完成隐含概率换算与高级数据修正</t>
+          <t>经模型综合分析：西甲，主胜概率领先客胜；风险中；已接入本次实时赔率快照，并完成隐含概率换算与高级数据修正；同场次已与竞彩足球 周六017 胜平负方向强制一致</t>
         </is>
       </c>
       <c r="AA114" t="inlineStr">
@@ -12511,13 +12511,13 @@
         </is>
       </c>
       <c r="K115">
-        <v>0.3999</v>
+        <v>0.4352</v>
       </c>
       <c r="L115">
-        <v>0.2717</v>
+        <v>0.2643</v>
       </c>
       <c r="M115">
-        <v>0.3284</v>
+        <v>0.3005</v>
       </c>
       <c r="N115">
         <v>0.3999</v>
@@ -12544,11 +12544,11 @@
       </c>
       <c r="U115" t="inlineStr">
         <is>
-          <t>高</t>
+          <t>中</t>
         </is>
       </c>
       <c r="V115">
-        <v>23.68</v>
+        <v>36.46</v>
       </c>
       <c r="W115" t="inlineStr">
         <is>
@@ -12563,7 +12563,7 @@
       </c>
       <c r="Z115" t="inlineStr">
         <is>
-          <t>经模型综合分析：荷乙，主胜概率领先客胜；风险高；已接入本次实时赔率快照，并完成隐含概率换算与高级数据修正</t>
+          <t>经模型综合分析：荷乙，主胜概率领先客胜；风险高；已接入本次实时赔率快照，并完成隐含概率换算与高级数据修正；同场次已与竞彩足球 周六015 胜平负方向强制一致</t>
         </is>
       </c>
       <c r="AA115" t="inlineStr">
@@ -12757,13 +12757,13 @@
         </is>
       </c>
       <c r="K117">
-        <v>0.443</v>
+        <v>0.4872</v>
       </c>
       <c r="L117">
-        <v>0.2916</v>
+        <v>0.2814</v>
       </c>
       <c r="M117">
-        <v>0.2655</v>
+        <v>0.2314</v>
       </c>
       <c r="N117">
         <v>0.443</v>
@@ -12794,7 +12794,7 @@
         </is>
       </c>
       <c r="V117">
-        <v>35.72</v>
+        <v>46.6</v>
       </c>
       <c r="W117" t="inlineStr">
         <is>
@@ -12809,7 +12809,7 @@
       </c>
       <c r="Z117" t="inlineStr">
         <is>
-          <t>经模型综合分析：瑞超，主胜概率领先平局；风险中；已接入本次实时赔率快照，并完成隐含概率换算与高级数据修正</t>
+          <t>经模型综合分析：瑞超，主胜概率领先平局；风险中；已接入本次实时赔率快照，并完成隐含概率换算与高级数据修正；同场次已与竞彩足球 周六007 胜平负方向强制一致</t>
         </is>
       </c>
       <c r="AA117" t="inlineStr">
@@ -12856,7 +12856,7 @@
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>平局</t>
+          <t>客胜</t>
         </is>
       </c>
       <c r="G118" t="inlineStr">
@@ -12866,7 +12866,7 @@
       </c>
       <c r="H118" t="inlineStr">
         <is>
-          <t>2-2</t>
+          <t>1-2</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -12876,17 +12876,17 @@
       </c>
       <c r="J118" t="inlineStr">
         <is>
-          <t>主胜-平局</t>
+          <t>主胜-客胜</t>
         </is>
       </c>
       <c r="K118">
-        <v>0.521</v>
+        <v>0.5009</v>
       </c>
       <c r="L118">
-        <v>0.2408</v>
+        <v>0.2465</v>
       </c>
       <c r="M118">
-        <v>0.2382</v>
+        <v>0.2526</v>
       </c>
       <c r="N118">
         <v>0.521</v>
@@ -12917,7 +12917,7 @@
         </is>
       </c>
       <c r="V118">
-        <v>52.93</v>
+        <v>51.41</v>
       </c>
       <c r="W118" t="inlineStr">
         <is>
@@ -12932,7 +12932,7 @@
       </c>
       <c r="Z118" t="inlineStr">
         <is>
-          <t>经模型综合分析：芬超，主胜概率领先平局；风险中；已接入本次实时赔率快照，并完成隐含概率换算与高级数据修正</t>
+          <t>经模型综合分析：芬超，主胜概率领先平局；风险中；已接入本次实时赔率快照，并完成隐含概率换算与高级数据修正；同场次已与竞彩足球 周六008 胜平负方向强制一致</t>
         </is>
       </c>
       <c r="AA118" t="inlineStr">
@@ -13003,13 +13003,13 @@
         </is>
       </c>
       <c r="K119">
-        <v>0.4923</v>
+        <v>0.4828</v>
       </c>
       <c r="L119">
-        <v>0.2635</v>
+        <v>0.272</v>
       </c>
       <c r="M119">
-        <v>0.2441</v>
+        <v>0.2452</v>
       </c>
       <c r="N119">
         <v>0.4923</v>
@@ -13040,7 +13040,7 @@
         </is>
       </c>
       <c r="V119">
-        <v>46.24</v>
+        <v>46.73</v>
       </c>
       <c r="W119" t="inlineStr">
         <is>
@@ -13055,7 +13055,7 @@
       </c>
       <c r="Z119" t="inlineStr">
         <is>
-          <t>经模型综合分析：芬超，主胜概率领先平局；风险中；已接入本次实时赔率快照，并完成隐含概率换算与高级数据修正</t>
+          <t>经模型综合分析：芬超，主胜概率领先平局；风险中；已接入本次实时赔率快照，并完成隐含概率换算与高级数据修正；同场次已与竞彩足球 周六011 胜平负方向强制一致</t>
         </is>
       </c>
       <c r="AA119" t="inlineStr">
@@ -13107,7 +13107,7 @@
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>2-1</t>
+          <t>3-1</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
@@ -13126,13 +13126,13 @@
         </is>
       </c>
       <c r="K120">
-        <v>0.5759</v>
+        <v>0.5934</v>
       </c>
       <c r="L120">
-        <v>0.2432</v>
+        <v>0.2361</v>
       </c>
       <c r="M120">
-        <v>0.181</v>
+        <v>0.1705</v>
       </c>
       <c r="N120">
         <v>0.5759</v>
@@ -13163,7 +13163,7 @@
         </is>
       </c>
       <c r="V120">
-        <v>61.61</v>
+        <v>67.88</v>
       </c>
       <c r="W120" t="inlineStr">
         <is>
@@ -13178,7 +13178,7 @@
       </c>
       <c r="Z120" t="inlineStr">
         <is>
-          <t>经模型综合分析：芬超，主胜概率领先平局；风险中；已接入本次实时赔率快照，并完成隐含概率换算与高级数据修正</t>
+          <t>经模型综合分析：芬超，主胜概率领先平局；风险中；已接入本次实时赔率快照，并完成隐含概率换算与高级数据修正；同场次已与竞彩足球 周六010 胜平负方向强制一致</t>
         </is>
       </c>
       <c r="AA120" t="inlineStr">
@@ -13249,13 +13249,13 @@
         </is>
       </c>
       <c r="K121">
-        <v>0.369</v>
+        <v>0.3731</v>
       </c>
       <c r="L121">
-        <v>0.2689</v>
+        <v>0.2676</v>
       </c>
       <c r="M121">
-        <v>0.362</v>
+        <v>0.3593</v>
       </c>
       <c r="N121">
         <v>0.369</v>
@@ -13286,7 +13286,7 @@
         </is>
       </c>
       <c r="V121">
-        <v>15.65</v>
+        <v>19.36</v>
       </c>
       <c r="W121" t="inlineStr">
         <is>
@@ -13301,7 +13301,7 @@
       </c>
       <c r="Z121" t="inlineStr">
         <is>
-          <t>经模型综合分析：芬超，主胜概率领先客胜；风险高；已接入本次实时赔率快照，并完成隐含概率换算与高级数据修正</t>
+          <t>经模型综合分析：芬超，主胜概率领先客胜；风险高；已接入本次实时赔率快照，并完成隐含概率换算与高级数据修正；同场次已与竞彩足球 周六009 胜平负方向强制一致</t>
         </is>
       </c>
       <c r="AA121" t="inlineStr">

</xml_diff>